<commit_message>
Table added, column sorted and cleaned
dim_date table added
dim_customer table's column sorted and cleaned
</commit_message>
<xml_diff>
--- a/Table Details.xlsx
+++ b/Table Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anmol\Desktop\Omkar_Data Analytics\GitHub\Onlineoffline sales data analysis\SQL Analysis Project  - Onlineoffline sales data analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A923102-4C66-4BBC-B2C4-F6EF3282E279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B66A68F-14B0-4F95-A4DE-E421C264BB24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A5A01D9C-68AD-4736-A120-B2455653887D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>dim_address</t>
   </si>
@@ -82,9 +82,6 @@
   </si>
   <si>
     <t>Done</t>
-  </si>
-  <si>
-    <t>Issue in colounmns</t>
   </si>
 </sst>
 </file>
@@ -504,7 +501,7 @@
         <v>1000</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">

</xml_diff>